<commit_message>
Complete API testing and update documentation
</commit_message>
<xml_diff>
--- a/bug-reports/Bug_Report.xlsx
+++ b/bug-reports/Bug_Report.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ecommerce-manual-testing\bug-reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C145F12F-4328-4138-9268-3E1518294F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB859B8B-38C7-4344-B62F-535512B16FE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0897DCB1-C57B-4B0E-B7C4-2D8C5854A411}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{0897DCB1-C57B-4B0E-B7C4-2D8C5854A411}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="UI" sheetId="1" r:id="rId1"/>
+    <sheet name="API" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="65">
   <si>
     <t>Bug ID</t>
   </si>
@@ -263,6 +264,34 @@
   </si>
   <si>
     <t>Staff vẫn truy cập được trang quản lý User bằng URL trực tiếp.</t>
+  </si>
+  <si>
+    <t>BUG_API_PRODUCT_001</t>
+  </si>
+  <si>
+    <t>API allows creating product with empty required Product Name</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Admin đã đăng nhập và có valid token</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Gửi POST /api/products 
+2. Để product_name trống 
+3. Các field required khác hợp lệ 
+4. Send  </t>
+  </si>
+  <si>
+    <t>API từ chối request và không tạo sản phẩm</t>
+  </si>
+  <si>
+    <t>API trả 201 Created và tạo sản phẩm với product_name="", slug=""</t>
+  </si>
+  <si>
+    <t>Case 1: product_name = [empty].
+Case 2: description = [empty].</t>
   </si>
 </sst>
 </file>
@@ -324,7 +353,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -350,6 +379,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1066,6 +1101,99 @@
         <a:xfrm>
           <a:off x="21549360" y="14339316"/>
           <a:ext cx="3651245" cy="1933237"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>60285</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2988304</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1644802</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E492ED1F-3319-6A9D-08CB-0D4F81DA4C15}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16450905" y="289560"/>
+          <a:ext cx="2928019" cy="1553362"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3119044</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>6127745</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1646594</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0657A515-62BC-DAEF-3735-2B75EBC69C41}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19509664" y="243840"/>
+          <a:ext cx="3008701" cy="1600874"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1816,4 +1944,440 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A97A0BAB-0535-480E-B8BD-9E76519FCF56}">
+  <dimension ref="A1:L26"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.88671875" customWidth="1"/>
+    <col min="2" max="2" width="24.109375" customWidth="1"/>
+    <col min="3" max="3" width="22.5546875" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" customWidth="1"/>
+    <col min="5" max="5" width="31.21875" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="7" width="20.6640625" customWidth="1"/>
+    <col min="8" max="8" width="21.77734375" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" customWidth="1"/>
+    <col min="10" max="10" width="10.77734375" customWidth="1"/>
+    <col min="11" max="11" width="11.88671875" customWidth="1"/>
+    <col min="12" max="12" width="90.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="133.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="4"/>
+    </row>
+    <row r="3" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+    </row>
+    <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+    </row>
+    <row r="5" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+    </row>
+    <row r="6" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+    </row>
+    <row r="7" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+    </row>
+    <row r="10" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+    </row>
+    <row r="11" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+    </row>
+    <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+    </row>
+    <row r="13" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+    </row>
+    <row r="14" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+    </row>
+    <row r="15" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+    </row>
+    <row r="16" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+    </row>
+    <row r="17" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+    </row>
+    <row r="18" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
+    </row>
+    <row r="19" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
+    </row>
+    <row r="20" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
+    </row>
+    <row r="21" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
+    </row>
+    <row r="22" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+    </row>
+    <row r="23" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+    </row>
+    <row r="24" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
+    </row>
+    <row r="25" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="11"/>
+    </row>
+    <row r="26" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="11"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="11"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>